<commit_message>
video 26 and yufa
</commit_message>
<xml_diff>
--- a/English/大雁单词.xlsx
+++ b/English/大雁单词.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data\study\web\Englidh\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data\study\Study\English\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51E25385-6AA3-480D-8357-918D0DACCE86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C13B7A60-1A63-4135-AC08-2D4DDD4BEF64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15264" yWindow="0" windowWidth="15552" windowHeight="16656" firstSheet="21" activeTab="25" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Video 1" sheetId="2" r:id="rId1"/>
@@ -38,7 +38,8 @@
     <sheet name="Video 23" sheetId="32" r:id="rId23"/>
     <sheet name="Video 24" sheetId="33" r:id="rId24"/>
     <sheet name="Video 25" sheetId="34" r:id="rId25"/>
-    <sheet name="Total 44" sheetId="13" r:id="rId26"/>
+    <sheet name="Video 26" sheetId="35" r:id="rId26"/>
+    <sheet name="Total 44" sheetId="13" r:id="rId27"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -61,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5111" uniqueCount="4164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5381" uniqueCount="4427">
   <si>
     <t>space</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -16715,6 +16716,1058 @@
   </si>
   <si>
     <t>n. 漏洞</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>cause</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 起因、理由、事业  v. 导致</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>due</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>adj. 由于、预期的、应得的  n. 应付款</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>duly</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>adv. 适当地、恰当地</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>given</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>adj. 规定的、特定的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ingredient</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 成分、材料、因素</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>element</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 要素、因素、基础</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>elementary</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>adj. 基本的、初级的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>factor</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 因素、要素</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>sake</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 缘故</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>forgive</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v. 原谅、免除</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>forgiving</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>adj. 宽宏大量的、宽容的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>curse</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v. 诅咒、咒骂  n. 咒骂</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>scold</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v. 责骂、训斥</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>accuse</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v. 控诉、控告、谴责</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>accusation</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 控告、谴责</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>excuse</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v. 原谅、免除  n. 借口</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>quarrel</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 争吵、吵架</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>quarrelsome</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>adj. 爱争吵的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>insult</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 辱骂、侮辱、冒犯</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>consult</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v. 咨询、请教</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>consultation</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 咨询</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>consultative</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>adj. 咨询的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>consultant</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>blame</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v. 责备、责怪  n. 责备</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>tame</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v. 驯服、制服  adj. 驯服的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>melt</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v. 融化</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>critic</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 批评家、评论家</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>criticise</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v. 批评</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>criticism</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 批评、批判</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>critical</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>adj. 决定性的、关键的、严重的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>criterion</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 标准、准则、原则</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>assist</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v. 帮助、促进</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>assistance</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 帮助、援助</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>assistant</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 助手、助理</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>resist</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v. 抵挡、抵制、阻挡</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>resistance</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 阻力、电阻、抵抗</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>insist</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v. 坚持、坚称</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>insistence</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 坚持</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>insistent</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>adj. 坚持的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>persist</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v. 坚持、继续存在</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>persistence</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>persistent</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>adj. 坚持的、持续的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>consist</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v. 由…组成、构成</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>comprise</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v. 包括、由…组成</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>praise</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 表扬、赞美</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>enterprise</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 企业、规划、事业</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>enterprising</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>adj. 有事业心的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>entrepreneur</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 企业家</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>entrepreneurial</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>adj. 创业的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>corporation</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 公司、法人</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>corporate</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>adj. 公司的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>empire</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 帝国、大企业</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>emperor</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 皇帝</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>empress</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 女皇</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>accompany</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v. 陪伴、伴随</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>companion</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 同伴、朋友</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>companionship</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 友情、友谊</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>manage</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v. 完成、解决、管理</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>management</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>manager</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 管理人员、经理</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>managerial</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>adj. 经理的、管理的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>chair</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 椅子、主席  v. 主持</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>chairman</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 主席、议长、会长</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>president</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 总统、主席、董事长</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>presidency</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 总统的职位</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>presidential</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>adj. 总统的、国家主席的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>harness</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v. 控制、利用</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>control</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v. 指挥、管理、控制</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>compete</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v. 参加比赛</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>competitor</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 竞争对手</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>competitive</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>adj. 竞争的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>competition</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>competent</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>adj. 有能力的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>complete</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v. 完成   adj. 完成的、彻底的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>completion</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 完成、结束</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>versus</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>对抗</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>crisis</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 危机</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>finance</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 资金、财政、金融</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>financial</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>adj. 财政的、金融的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>funding</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 专款、资金、提供资金</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>fund</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 基金、资金</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>commerce</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 贸易、商业</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>commercial</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>adj. 贸易的、赢利的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>commercialise</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v. 商业化</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>commodity</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 商品、有用的东西</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>goods</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 商品</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>merchant</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 商人、批发商</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>stock</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 库存、股票  v. 存货</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>storage</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 贮藏</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>trade</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 贸易 v. 做生意</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>trademark</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 商标</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>budget</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 预算</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>budgetary</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>adj. 预算的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>gadget</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 小玩意、小装置</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>gadgetry</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 小装置</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>target</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 目标、靶子  v. 瞄准</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>destination</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 目的地、终点、目标</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>revenue</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 收入、收益</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>avenue</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 大街、途径、手段</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>income</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>gross</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>adj. 总的、毛的、严重的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>economy</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 经济、国家</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>economic</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>adj. 经济学的、可赚钱的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>economics</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 经济学、经济情况</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>economist</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 经济学家</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>economical</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>adj. 经济的、节俭的、节约的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>scientific</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>adj. 科学上的、细致严谨的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>science</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 科学</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>scientist</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 科学家</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>evil</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>adj. 恶毒的、邪恶的  n. 邪恶</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>produce</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v. 生产、制造、展现</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>product</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 产物、产品</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>production</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 生产、制造、制作</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>productive</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>adj. 生产的、有效益的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>reproduce</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v. 复制、再生产</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>reproduction</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 生殖、繁衍</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>reproductive</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>adj. 繁殖的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>productivity</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 生产率、生产力</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>industry</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 工业、行业、勤奋</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>industrial</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>adj. 工业的、产业的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>industrialize</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v. 工业化</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>industrious</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>adj. 勤奋的、勤劳的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>manipulate</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v. 操作、操纵、影响</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>manipulation</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 控制、操纵</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>manipulative</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>adj. 善于控制的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>operate</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v. 运作、工作、操作</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>operator</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 操作人员</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>operation</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 手术</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>operational</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>adj. 操作的、运转的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>cooperate</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v. 合作、协作</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>cooperation</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>n. 合作、协作</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>cooperative</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>adj. 合作的、同心协力的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>collaborate</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>collaboration</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>collaborative</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>adj. 合作的、协作的</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -35367,6 +36420,1100 @@
 </file>
 
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54EBE5E2-80D0-4BB8-A544-C7F5CF55B910}">
+  <dimension ref="A1:B135"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="19.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>4164</v>
+      </c>
+      <c r="B1" t="s">
+        <v>4165</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>4166</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4167</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>4168</v>
+      </c>
+      <c r="B3" t="s">
+        <v>4169</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>4170</v>
+      </c>
+      <c r="B4" t="s">
+        <v>4171</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>4172</v>
+      </c>
+      <c r="B5" t="s">
+        <v>4173</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>4174</v>
+      </c>
+      <c r="B6" t="s">
+        <v>4175</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>4176</v>
+      </c>
+      <c r="B7" t="s">
+        <v>4177</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>4178</v>
+      </c>
+      <c r="B8" t="s">
+        <v>4179</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>4180</v>
+      </c>
+      <c r="B9" t="s">
+        <v>4181</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>4182</v>
+      </c>
+      <c r="B10" t="s">
+        <v>4183</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>4184</v>
+      </c>
+      <c r="B11" t="s">
+        <v>4185</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>4186</v>
+      </c>
+      <c r="B12" t="s">
+        <v>4187</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>4188</v>
+      </c>
+      <c r="B13" t="s">
+        <v>4189</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>4190</v>
+      </c>
+      <c r="B14" t="s">
+        <v>4191</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>4192</v>
+      </c>
+      <c r="B15" t="s">
+        <v>4193</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>4194</v>
+      </c>
+      <c r="B16" t="s">
+        <v>4195</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>4196</v>
+      </c>
+      <c r="B17" t="s">
+        <v>4197</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>4198</v>
+      </c>
+      <c r="B18" t="s">
+        <v>4199</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>4200</v>
+      </c>
+      <c r="B19" t="s">
+        <v>4201</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>4202</v>
+      </c>
+      <c r="B20" t="s">
+        <v>4203</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>4204</v>
+      </c>
+      <c r="B21" t="s">
+        <v>4205</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>4206</v>
+      </c>
+      <c r="B22" t="s">
+        <v>4207</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>4208</v>
+      </c>
+      <c r="B23" t="s">
+        <v>2777</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>4209</v>
+      </c>
+      <c r="B24" t="s">
+        <v>4210</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>4211</v>
+      </c>
+      <c r="B25" t="s">
+        <v>4212</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>4213</v>
+      </c>
+      <c r="B26" t="s">
+        <v>4214</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>4215</v>
+      </c>
+      <c r="B27" t="s">
+        <v>4216</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>4217</v>
+      </c>
+      <c r="B28" t="s">
+        <v>4218</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>4219</v>
+      </c>
+      <c r="B29" t="s">
+        <v>4220</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>4221</v>
+      </c>
+      <c r="B30" t="s">
+        <v>4222</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>4223</v>
+      </c>
+      <c r="B31" t="s">
+        <v>4224</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>4225</v>
+      </c>
+      <c r="B32" t="s">
+        <v>4226</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>4227</v>
+      </c>
+      <c r="B33" t="s">
+        <v>4228</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>4229</v>
+      </c>
+      <c r="B34" t="s">
+        <v>4230</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>4231</v>
+      </c>
+      <c r="B35" t="s">
+        <v>4232</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>4233</v>
+      </c>
+      <c r="B36" t="s">
+        <v>4234</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>4235</v>
+      </c>
+      <c r="B37" t="s">
+        <v>4236</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>4237</v>
+      </c>
+      <c r="B38" t="s">
+        <v>4238</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>4239</v>
+      </c>
+      <c r="B39" t="s">
+        <v>4240</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>4241</v>
+      </c>
+      <c r="B40" t="s">
+        <v>4242</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>4243</v>
+      </c>
+      <c r="B41" t="s">
+        <v>4238</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>4244</v>
+      </c>
+      <c r="B42" t="s">
+        <v>4245</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>4246</v>
+      </c>
+      <c r="B43" t="s">
+        <v>4247</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>4248</v>
+      </c>
+      <c r="B44" t="s">
+        <v>4249</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>4250</v>
+      </c>
+      <c r="B45" t="s">
+        <v>4251</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>4252</v>
+      </c>
+      <c r="B46" t="s">
+        <v>4253</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>4254</v>
+      </c>
+      <c r="B47" t="s">
+        <v>4255</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>4256</v>
+      </c>
+      <c r="B48" t="s">
+        <v>4257</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>4258</v>
+      </c>
+      <c r="B49" t="s">
+        <v>4259</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>4260</v>
+      </c>
+      <c r="B50" t="s">
+        <v>4261</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>4262</v>
+      </c>
+      <c r="B51" t="s">
+        <v>4263</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>4264</v>
+      </c>
+      <c r="B52" t="s">
+        <v>4265</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>4266</v>
+      </c>
+      <c r="B53" t="s">
+        <v>4267</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>4268</v>
+      </c>
+      <c r="B54" t="s">
+        <v>4269</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>4270</v>
+      </c>
+      <c r="B55" t="s">
+        <v>4271</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>4272</v>
+      </c>
+      <c r="B56" t="s">
+        <v>4273</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>4274</v>
+      </c>
+      <c r="B57" t="s">
+        <v>4275</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>4276</v>
+      </c>
+      <c r="B58" t="s">
+        <v>4277</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>4278</v>
+      </c>
+      <c r="B59" t="s">
+        <v>859</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>4279</v>
+      </c>
+      <c r="B60" t="s">
+        <v>4280</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>4281</v>
+      </c>
+      <c r="B61" t="s">
+        <v>4282</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>4283</v>
+      </c>
+      <c r="B62" t="s">
+        <v>4284</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>4285</v>
+      </c>
+      <c r="B63" t="s">
+        <v>4286</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>4287</v>
+      </c>
+      <c r="B64" t="s">
+        <v>4288</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>4289</v>
+      </c>
+      <c r="B65" t="s">
+        <v>4290</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>4291</v>
+      </c>
+      <c r="B66" t="s">
+        <v>4292</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>4293</v>
+      </c>
+      <c r="B67" t="s">
+        <v>4294</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>4295</v>
+      </c>
+      <c r="B68" t="s">
+        <v>4296</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>4297</v>
+      </c>
+      <c r="B69" t="s">
+        <v>4298</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>4299</v>
+      </c>
+      <c r="B70" t="s">
+        <v>4300</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>4301</v>
+      </c>
+      <c r="B71" t="s">
+        <v>4302</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>4303</v>
+      </c>
+      <c r="B72" t="s">
+        <v>2905</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>4304</v>
+      </c>
+      <c r="B73" t="s">
+        <v>4305</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>4306</v>
+      </c>
+      <c r="B74" t="s">
+        <v>4307</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>4308</v>
+      </c>
+      <c r="B75" t="s">
+        <v>4309</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>4310</v>
+      </c>
+      <c r="B76" t="s">
+        <v>4311</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>4312</v>
+      </c>
+      <c r="B77" t="s">
+        <v>4313</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>4314</v>
+      </c>
+      <c r="B78" t="s">
+        <v>4315</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>4316</v>
+      </c>
+      <c r="B79" t="s">
+        <v>4317</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>4318</v>
+      </c>
+      <c r="B80" t="s">
+        <v>4319</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>4320</v>
+      </c>
+      <c r="B81" t="s">
+        <v>4321</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>4322</v>
+      </c>
+      <c r="B82" t="s">
+        <v>4323</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>4324</v>
+      </c>
+      <c r="B83" t="s">
+        <v>4325</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>4326</v>
+      </c>
+      <c r="B84" t="s">
+        <v>4327</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>4328</v>
+      </c>
+      <c r="B85" t="s">
+        <v>4329</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>4330</v>
+      </c>
+      <c r="B86" t="s">
+        <v>4331</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>4332</v>
+      </c>
+      <c r="B87" t="s">
+        <v>4333</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>4334</v>
+      </c>
+      <c r="B88" t="s">
+        <v>4335</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>4336</v>
+      </c>
+      <c r="B89" t="s">
+        <v>4337</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>4338</v>
+      </c>
+      <c r="B90" t="s">
+        <v>4339</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>4340</v>
+      </c>
+      <c r="B91" t="s">
+        <v>4341</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>4342</v>
+      </c>
+      <c r="B92" t="s">
+        <v>4343</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>4344</v>
+      </c>
+      <c r="B93" t="s">
+        <v>4345</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>4346</v>
+      </c>
+      <c r="B94" t="s">
+        <v>4347</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>4348</v>
+      </c>
+      <c r="B95" t="s">
+        <v>4349</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>4350</v>
+      </c>
+      <c r="B96" t="s">
+        <v>4351</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>4352</v>
+      </c>
+      <c r="B97" t="s">
+        <v>4353</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>4354</v>
+      </c>
+      <c r="B98" t="s">
+        <v>4355</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>4356</v>
+      </c>
+      <c r="B99" t="s">
+        <v>4357</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>4358</v>
+      </c>
+      <c r="B100" t="s">
+        <v>4355</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>4359</v>
+      </c>
+      <c r="B101" t="s">
+        <v>4360</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>4361</v>
+      </c>
+      <c r="B102" t="s">
+        <v>4362</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>4363</v>
+      </c>
+      <c r="B103" t="s">
+        <v>4364</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>4365</v>
+      </c>
+      <c r="B104" t="s">
+        <v>4366</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>4367</v>
+      </c>
+      <c r="B105" t="s">
+        <v>4368</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>4369</v>
+      </c>
+      <c r="B106" t="s">
+        <v>4370</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>4371</v>
+      </c>
+      <c r="B107" t="s">
+        <v>4372</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>4373</v>
+      </c>
+      <c r="B108" t="s">
+        <v>4374</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>4375</v>
+      </c>
+      <c r="B109" t="s">
+        <v>4376</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>4377</v>
+      </c>
+      <c r="B110" t="s">
+        <v>4378</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>4379</v>
+      </c>
+      <c r="B111" t="s">
+        <v>4380</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>4381</v>
+      </c>
+      <c r="B112" t="s">
+        <v>4382</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>4383</v>
+      </c>
+      <c r="B113" t="s">
+        <v>4384</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>4385</v>
+      </c>
+      <c r="B114" t="s">
+        <v>4386</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>4387</v>
+      </c>
+      <c r="B115" t="s">
+        <v>4388</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>4389</v>
+      </c>
+      <c r="B116" t="s">
+        <v>4390</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>4391</v>
+      </c>
+      <c r="B117" t="s">
+        <v>4392</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>4393</v>
+      </c>
+      <c r="B118" t="s">
+        <v>4394</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>4395</v>
+      </c>
+      <c r="B119" t="s">
+        <v>4396</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>4397</v>
+      </c>
+      <c r="B120" t="s">
+        <v>4398</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>4399</v>
+      </c>
+      <c r="B121" t="s">
+        <v>4400</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>4401</v>
+      </c>
+      <c r="B122" t="s">
+        <v>4402</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>4403</v>
+      </c>
+      <c r="B123" t="s">
+        <v>4404</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>4405</v>
+      </c>
+      <c r="B124" t="s">
+        <v>4406</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>4407</v>
+      </c>
+      <c r="B125" t="s">
+        <v>4408</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
+        <v>4409</v>
+      </c>
+      <c r="B126" t="s">
+        <v>4410</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A127" t="s">
+        <v>4411</v>
+      </c>
+      <c r="B127" t="s">
+        <v>4412</v>
+      </c>
+    </row>
+    <row r="128" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A128" t="s">
+        <v>4413</v>
+      </c>
+      <c r="B128" t="s">
+        <v>4414</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A129" t="s">
+        <v>4415</v>
+      </c>
+      <c r="B129" t="s">
+        <v>4416</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A130" t="s">
+        <v>4417</v>
+      </c>
+      <c r="B130" t="s">
+        <v>4418</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A131" t="s">
+        <v>4419</v>
+      </c>
+      <c r="B131" t="s">
+        <v>4420</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A132" t="s">
+        <v>4421</v>
+      </c>
+      <c r="B132" t="s">
+        <v>4422</v>
+      </c>
+    </row>
+    <row r="133" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A133" t="s">
+        <v>4423</v>
+      </c>
+      <c r="B133" t="s">
+        <v>4418</v>
+      </c>
+    </row>
+    <row r="134" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A134" t="s">
+        <v>4424</v>
+      </c>
+      <c r="B134" t="s">
+        <v>4420</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A135" t="s">
+        <v>4425</v>
+      </c>
+      <c r="B135" t="s">
+        <v>4426</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A35902E0-5DA8-4F9A-A665-EE84FD306EF5}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>

</xml_diff>